<commit_message>
Update gitignore to ignore Python cache files
</commit_message>
<xml_diff>
--- a/reports/excel/overall/low_psh_generation_report_19-05-2026.xlsx
+++ b/reports/excel/overall/low_psh_generation_report_19-05-2026.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -502,37 +502,37 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plant Name</t>
+          <t>PLANT NAME</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>STATUS</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total Capacity (kWp)</t>
+          <t>TOTAL CAPACITY (KWP)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Grid Connected Date</t>
+          <t>GRID CONNECTION DATE</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Inverter Name</t>
+          <t>INVERTER NAME</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Inverter SN</t>
+          <t>INVERTER SN</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>String Number</t>
+          <t>STRING NUMBER</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>6T21A9037832</t>
+          <t>NE=50476040</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BP PLASTICS HQ</t>
+          <t>DSG MALAYSIA SDN. BHD</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -674,39 +674,61 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1063.425</v>
+        <v>2310.255</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2025-01-16</t>
+          <t>2022-11-24</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Inverter_1</t>
+          <t>100KTL-M1(COM1-11)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>6T2479016090</t>
+          <t>NE=50412015</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KWANG HUA PERSENDIRIAN  METER  2-3-4-5-6</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>302.475</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2022-03-04</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Block C - Inverter 7 - Meter 2</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>NE=51163025</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -719,20 +741,42 @@
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>PKT 12 WAVES</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1337.31</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-05</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 1</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003099</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -745,7 +789,7 @@
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -758,7 +802,7 @@
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -767,19 +811,11 @@
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Inverter_7</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>6T2479016026</t>
-        </is>
-      </c>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -805,7 +841,7 @@
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -818,7 +854,7 @@
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -831,7 +867,7 @@
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -840,11 +876,19 @@
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 10</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003102</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -857,7 +901,7 @@
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -870,7 +914,7 @@
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -879,89 +923,37 @@
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="4" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Inverter_9</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>ES2460041537</t>
-        </is>
-      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>DSG MALAYSIA SDN. BHD</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>2310.255</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>2022-11-24</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>100KTL-M1(COM1-1)</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>6T21A9013292</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>KWANG HUA PERSENDIRIAN  METER  2-3-4-5-6</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>302.475</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2022-03-04</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Block B2-Inverter 6 - Meter 6</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>6T21C9025214</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -974,7 +966,7 @@
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -987,7 +979,7 @@
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -996,19 +988,11 @@
       <c r="B29" s="4" t="n"/>
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="4" t="n"/>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Block C - Inverter 7 - Meter 2</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>6T21C9024903</t>
-        </is>
-      </c>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PV 1 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1021,42 +1005,28 @@
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>QL FOODS</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>2061.225</v>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>2024-10-03</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>INVERTER _5 R1</t>
+          <t>Inverter 2</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>6T24A9031290</t>
+          <t>NE=56003098</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1039,7 @@
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1065,7 @@
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1078,7 @@
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1091,7 @@
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1104,7 @@
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1143,11 +1113,19 @@
       <c r="B38" s="4" t="n"/>
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 3</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003101</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1138,7 @@
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1151,7 @@
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1164,7 @@
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1177,7 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1208,11 +1186,19 @@
       <c r="B43" s="4" t="n"/>
       <c r="C43" s="4" t="n"/>
       <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 4</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003104</t>
+        </is>
+      </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1211,7 @@
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1224,7 @@
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1237,7 @@
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1250,7 @@
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1263,7 @@
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1286,19 +1272,11 @@
       <c r="B49" s="4" t="n"/>
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="4" t="n"/>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_1</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055730</t>
-        </is>
-      </c>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1289,7 @@
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1302,7 @@
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1333,11 +1311,19 @@
       <c r="B52" s="4" t="n"/>
       <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 5</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003103</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1336,7 @@
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1349,7 @@
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1375,7 @@
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1388,7 @@
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1401,7 @@
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1414,7 @@
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1427,7 @@
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1450,11 +1436,19 @@
       <c r="B61" s="4" t="n"/>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="4" t="n"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 6</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003095</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1461,7 @@
       <c r="F62" s="4" t="n"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1474,7 @@
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1487,7 @@
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1500,7 @@
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1515,11 +1509,19 @@
       <c r="B66" s="4" t="n"/>
       <c r="C66" s="4" t="n"/>
       <c r="D66" s="4" t="n"/>
-      <c r="E66" s="4" t="n"/>
-      <c r="F66" s="4" t="n"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 7</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003100</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1534,7 @@
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1541,19 +1543,11 @@
       <c r="B68" s="4" t="n"/>
       <c r="C68" s="4" t="n"/>
       <c r="D68" s="4" t="n"/>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_10</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>6T2449032177</t>
-        </is>
-      </c>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1560,7 @@
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1573,7 @@
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1586,7 @@
       <c r="F71" s="4" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1601,19 +1595,11 @@
       <c r="B72" s="4" t="n"/>
       <c r="C72" s="4" t="n"/>
       <c r="D72" s="4" t="n"/>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_12</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055893</t>
-        </is>
-      </c>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1622,11 +1608,19 @@
       <c r="B73" s="4" t="n"/>
       <c r="C73" s="4" t="n"/>
       <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
-      <c r="F73" s="4" t="n"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 8</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003096</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1633,7 @@
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1646,7 @@
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1659,7 @@
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1672,7 @@
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1685,7 @@
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1698,7 @@
       <c r="F79" s="4" t="n"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1707,19 @@
       <c r="B80" s="4" t="n"/>
       <c r="C80" s="4" t="n"/>
       <c r="D80" s="4" t="n"/>
-      <c r="E80" s="4" t="n"/>
-      <c r="F80" s="4" t="n"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Inverter 9</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>NE=56003097</t>
+        </is>
+      </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1732,7 @@
       <c r="F81" s="4" t="n"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1745,7 @@
       <c r="F82" s="4" t="n"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1758,7 @@
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1771,7 @@
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1784,7 @@
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1808,20 +1810,42 @@
       <c r="F87" s="4" t="n"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="4" t="n"/>
-      <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="n"/>
-      <c r="D88" s="4" t="n"/>
-      <c r="E88" s="4" t="n"/>
-      <c r="F88" s="4" t="n"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>QL FOODS</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>2061.225</v>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2024-10-03</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER _5 R1</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>NE=54942978</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1858,7 @@
       <c r="F89" s="4" t="n"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1871,7 @@
       <c r="F90" s="4" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1856,19 +1880,11 @@
       <c r="B91" s="4" t="n"/>
       <c r="C91" s="4" t="n"/>
       <c r="D91" s="4" t="n"/>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_13</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>6T2459004848</t>
-        </is>
-      </c>
+      <c r="E91" s="4" t="n"/>
+      <c r="F91" s="4" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>PV 1 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1897,7 @@
       <c r="F92" s="4" t="n"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1910,7 @@
       <c r="F93" s="4" t="n"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1923,7 @@
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1936,7 @@
       <c r="F95" s="4" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1949,7 @@
       <c r="F96" s="4" t="n"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1962,7 @@
       <c r="F97" s="4" t="n"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1975,7 @@
       <c r="F98" s="4" t="n"/>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 13 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1988,7 @@
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1985,7 +2001,7 @@
       <c r="F100" s="4" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2014,7 @@
       <c r="F101" s="4" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2027,7 @@
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2040,7 @@
       <c r="F103" s="4" t="n"/>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2053,7 @@
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2066,7 @@
       <c r="F105" s="4" t="n"/>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2059,11 +2075,19 @@
       <c r="B106" s="4" t="n"/>
       <c r="C106" s="4" t="n"/>
       <c r="D106" s="4" t="n"/>
-      <c r="E106" s="4" t="n"/>
-      <c r="F106" s="4" t="n"/>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_1</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>NE=53678484</t>
+        </is>
+      </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2100,7 @@
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2113,7 @@
       <c r="F108" s="4" t="n"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2126,7 @@
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2111,19 +2135,11 @@
       <c r="B110" s="4" t="n"/>
       <c r="C110" s="4" t="n"/>
       <c r="D110" s="4" t="n"/>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_14</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055894</t>
-        </is>
-      </c>
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="n"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2152,7 @@
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2165,7 @@
       <c r="F112" s="4" t="n"/>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2178,7 @@
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2191,7 @@
       <c r="F114" s="4" t="n"/>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2204,7 @@
       <c r="F115" s="4" t="n"/>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2217,7 @@
       <c r="F116" s="4" t="n"/>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2230,7 @@
       <c r="F117" s="4" t="n"/>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 13 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2243,7 @@
       <c r="F118" s="4" t="n"/>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2256,7 @@
       <c r="F119" s="4" t="n"/>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2269,7 @@
       <c r="F120" s="4" t="n"/>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2282,7 @@
       <c r="F121" s="4" t="n"/>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2295,7 @@
       <c r="F122" s="4" t="n"/>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2308,7 @@
       <c r="F123" s="4" t="n"/>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2321,7 @@
       <c r="F124" s="4" t="n"/>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2314,11 +2330,19 @@
       <c r="B125" s="4" t="n"/>
       <c r="C125" s="4" t="n"/>
       <c r="D125" s="4" t="n"/>
-      <c r="E125" s="4" t="n"/>
-      <c r="F125" s="4" t="n"/>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_10</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679611</t>
+        </is>
+      </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2355,7 @@
       <c r="F126" s="4" t="n"/>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2368,7 @@
       <c r="F127" s="4" t="n"/>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2381,7 @@
       <c r="F128" s="4" t="n"/>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2366,19 +2390,11 @@
       <c r="B129" s="4" t="n"/>
       <c r="C129" s="4" t="n"/>
       <c r="D129" s="4" t="n"/>
-      <c r="E129" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_15</t>
-        </is>
-      </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t>6T2449022635</t>
-        </is>
-      </c>
+      <c r="E129" s="4" t="n"/>
+      <c r="F129" s="4" t="n"/>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2407,7 @@
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2400,11 +2416,19 @@
       <c r="B131" s="4" t="n"/>
       <c r="C131" s="4" t="n"/>
       <c r="D131" s="4" t="n"/>
-      <c r="E131" s="4" t="n"/>
-      <c r="F131" s="4" t="n"/>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_12</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679581</t>
+        </is>
+      </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2441,7 @@
       <c r="F132" s="4" t="n"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2454,7 @@
       <c r="F133" s="4" t="n"/>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2467,7 @@
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2452,19 +2476,11 @@
       <c r="B135" s="4" t="n"/>
       <c r="C135" s="4" t="n"/>
       <c r="D135" s="4" t="n"/>
-      <c r="E135" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_2</t>
-        </is>
-      </c>
-      <c r="F135" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055797</t>
-        </is>
-      </c>
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="n"/>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2493,7 @@
       <c r="F136" s="4" t="n"/>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2506,7 @@
       <c r="F137" s="4" t="n"/>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2519,7 @@
       <c r="F138" s="4" t="n"/>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2532,7 @@
       <c r="F139" s="4" t="n"/>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2545,7 @@
       <c r="F140" s="4" t="n"/>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2558,7 @@
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2571,7 @@
       <c r="F142" s="4" t="n"/>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 13 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2584,7 @@
       <c r="F143" s="4" t="n"/>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2597,7 @@
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2610,7 @@
       <c r="F145" s="4" t="n"/>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2623,7 @@
       <c r="F146" s="4" t="n"/>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2636,7 @@
       <c r="F147" s="4" t="n"/>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2649,7 @@
       <c r="F148" s="4" t="n"/>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2662,7 @@
       <c r="F149" s="4" t="n"/>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2655,11 +2671,19 @@
       <c r="B150" s="4" t="n"/>
       <c r="C150" s="4" t="n"/>
       <c r="D150" s="4" t="n"/>
-      <c r="E150" s="4" t="n"/>
-      <c r="F150" s="4" t="n"/>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_13</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679495</t>
+        </is>
+      </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 1 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2696,7 @@
       <c r="F151" s="4" t="n"/>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2709,7 @@
       <c r="F152" s="4" t="n"/>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2722,7 @@
       <c r="F153" s="4" t="n"/>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2707,19 +2731,11 @@
       <c r="B154" s="4" t="n"/>
       <c r="C154" s="4" t="n"/>
       <c r="D154" s="4" t="n"/>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_3</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055789</t>
-        </is>
-      </c>
+      <c r="E154" s="4" t="n"/>
+      <c r="F154" s="4" t="n"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2748,7 @@
       <c r="F155" s="4" t="n"/>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2761,7 @@
       <c r="F156" s="4" t="n"/>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2774,7 @@
       <c r="F157" s="4" t="n"/>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2800,7 @@
       <c r="F159" s="4" t="n"/>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2813,7 @@
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2826,7 @@
       <c r="F161" s="4" t="n"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 13 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2839,7 @@
       <c r="F162" s="4" t="n"/>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2852,7 @@
       <c r="F163" s="4" t="n"/>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2845,19 +2861,11 @@
       <c r="B164" s="4" t="n"/>
       <c r="C164" s="4" t="n"/>
       <c r="D164" s="4" t="n"/>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_4</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055824</t>
-        </is>
-      </c>
+      <c r="E164" s="4" t="n"/>
+      <c r="F164" s="4" t="n"/>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2878,7 @@
       <c r="F165" s="4" t="n"/>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2879,19 +2887,11 @@
       <c r="B166" s="4" t="n"/>
       <c r="C166" s="4" t="n"/>
       <c r="D166" s="4" t="n"/>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_6</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055762</t>
-        </is>
-      </c>
+      <c r="E166" s="4" t="n"/>
+      <c r="F166" s="4" t="n"/>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       <c r="F167" s="4" t="n"/>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       <c r="F168" s="4" t="n"/>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2926,11 +2926,19 @@
       <c r="B169" s="4" t="n"/>
       <c r="C169" s="4" t="n"/>
       <c r="D169" s="4" t="n"/>
-      <c r="E169" s="4" t="n"/>
-      <c r="F169" s="4" t="n"/>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_14</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679493</t>
+        </is>
+      </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2951,7 @@
       <c r="F170" s="4" t="n"/>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2964,7 @@
       <c r="F171" s="4" t="n"/>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2977,7 @@
       <c r="F172" s="4" t="n"/>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2990,7 @@
       <c r="F173" s="4" t="n"/>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -2995,7 +3003,7 @@
       <c r="F174" s="4" t="n"/>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 7 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3016,7 @@
       <c r="F175" s="4" t="n"/>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3029,7 @@
       <c r="F176" s="4" t="n"/>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 9 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3042,7 @@
       <c r="F177" s="4" t="n"/>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>PV 19 Current (A) String</t>
+          <t>PV 10 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3055,7 @@
       <c r="F178" s="4" t="n"/>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>PV 20 Current (A) String</t>
+          <t>PV 11 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3056,19 +3064,11 @@
       <c r="B179" s="4" t="n"/>
       <c r="C179" s="4" t="n"/>
       <c r="D179" s="4" t="n"/>
-      <c r="E179" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_7</t>
-        </is>
-      </c>
-      <c r="F179" s="2" t="inlineStr">
-        <is>
-          <t>6T22A9046723</t>
-        </is>
-      </c>
+      <c r="E179" s="4" t="n"/>
+      <c r="F179" s="4" t="n"/>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 12 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       <c r="F180" s="4" t="n"/>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>PV 5 Current (A) String</t>
+          <t>PV 13 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       <c r="F181" s="4" t="n"/>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 14 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3103,19 +3103,11 @@
       <c r="B182" s="4" t="n"/>
       <c r="C182" s="4" t="n"/>
       <c r="D182" s="4" t="n"/>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>INVERTER_9</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>ES23C0055915</t>
-        </is>
-      </c>
+      <c r="E182" s="4" t="n"/>
+      <c r="F182" s="4" t="n"/>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>PV 1 Current (A) String</t>
+          <t>PV 15 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3120,7 @@
       <c r="F183" s="4" t="n"/>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>PV 2 Current (A) String</t>
+          <t>PV 16 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3133,7 @@
       <c r="F184" s="4" t="n"/>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>PV 3 Current (A) String</t>
+          <t>PV 17 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3146,7 @@
       <c r="F185" s="4" t="n"/>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>PV 4 Current (A) String</t>
+          <t>PV 18 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3159,7 @@
       <c r="F186" s="4" t="n"/>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>PV 6 Current (A) String</t>
+          <t>PV 19 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3172,7 @@
       <c r="F187" s="4" t="n"/>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>PV 7 Current (A) String</t>
+          <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3189,11 +3181,19 @@
       <c r="B188" s="4" t="n"/>
       <c r="C188" s="4" t="n"/>
       <c r="D188" s="4" t="n"/>
-      <c r="E188" s="4" t="n"/>
-      <c r="F188" s="4" t="n"/>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_15</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679053</t>
+        </is>
+      </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>PV 8 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       <c r="F189" s="4" t="n"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>PV 9 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       <c r="F190" s="4" t="n"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>PV 10 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       <c r="F191" s="4" t="n"/>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>PV 11 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3245,7 @@
       <c r="F192" s="4" t="n"/>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>PV 12 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       <c r="F193" s="4" t="n"/>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>PV 13 Current (A) String</t>
+          <t>PV 8 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3267,11 +3267,19 @@
       <c r="B194" s="4" t="n"/>
       <c r="C194" s="4" t="n"/>
       <c r="D194" s="4" t="n"/>
-      <c r="E194" s="4" t="n"/>
-      <c r="F194" s="4" t="n"/>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_2</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>NE=53678485</t>
+        </is>
+      </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>PV 14 Current (A) String</t>
+          <t>PV 2 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3292,7 @@
       <c r="F195" s="4" t="n"/>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>PV 15 Current (A) String</t>
+          <t>PV 3 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3305,7 @@
       <c r="F196" s="4" t="n"/>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>PV 16 Current (A) String</t>
+          <t>PV 4 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3318,7 @@
       <c r="F197" s="4" t="n"/>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>PV 17 Current (A) String</t>
+          <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3331,7 @@
       <c r="F198" s="4" t="n"/>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>PV 18 Current (A) String</t>
+          <t>PV 6 Current (A) String</t>
         </is>
       </c>
     </row>
@@ -3336,93 +3344,885 @@
       <c r="F199" s="4" t="n"/>
       <c r="G199" s="2" t="inlineStr">
         <is>
+          <t>PV 7 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="22" customHeight="1">
+      <c r="A200" s="4" t="n"/>
+      <c r="B200" s="4" t="n"/>
+      <c r="C200" s="4" t="n"/>
+      <c r="D200" s="4" t="n"/>
+      <c r="E200" s="4" t="n"/>
+      <c r="F200" s="4" t="n"/>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>PV 8 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="22" customHeight="1">
+      <c r="A201" s="4" t="n"/>
+      <c r="B201" s="4" t="n"/>
+      <c r="C201" s="4" t="n"/>
+      <c r="D201" s="4" t="n"/>
+      <c r="E201" s="4" t="n"/>
+      <c r="F201" s="4" t="n"/>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>PV 9 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="22" customHeight="1">
+      <c r="A202" s="4" t="n"/>
+      <c r="B202" s="4" t="n"/>
+      <c r="C202" s="4" t="n"/>
+      <c r="D202" s="4" t="n"/>
+      <c r="E202" s="4" t="n"/>
+      <c r="F202" s="4" t="n"/>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>PV 10 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="22" customHeight="1">
+      <c r="A203" s="4" t="n"/>
+      <c r="B203" s="4" t="n"/>
+      <c r="C203" s="4" t="n"/>
+      <c r="D203" s="4" t="n"/>
+      <c r="E203" s="4" t="n"/>
+      <c r="F203" s="4" t="n"/>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>PV 11 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="22" customHeight="1">
+      <c r="A204" s="4" t="n"/>
+      <c r="B204" s="4" t="n"/>
+      <c r="C204" s="4" t="n"/>
+      <c r="D204" s="4" t="n"/>
+      <c r="E204" s="4" t="n"/>
+      <c r="F204" s="4" t="n"/>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>PV 12 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="22" customHeight="1">
+      <c r="A205" s="4" t="n"/>
+      <c r="B205" s="4" t="n"/>
+      <c r="C205" s="4" t="n"/>
+      <c r="D205" s="4" t="n"/>
+      <c r="E205" s="4" t="n"/>
+      <c r="F205" s="4" t="n"/>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>PV 13 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="22" customHeight="1">
+      <c r="A206" s="4" t="n"/>
+      <c r="B206" s="4" t="n"/>
+      <c r="C206" s="4" t="n"/>
+      <c r="D206" s="4" t="n"/>
+      <c r="E206" s="4" t="n"/>
+      <c r="F206" s="4" t="n"/>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>PV 14 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="22" customHeight="1">
+      <c r="A207" s="4" t="n"/>
+      <c r="B207" s="4" t="n"/>
+      <c r="C207" s="4" t="n"/>
+      <c r="D207" s="4" t="n"/>
+      <c r="E207" s="4" t="n"/>
+      <c r="F207" s="4" t="n"/>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>PV 15 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="22" customHeight="1">
+      <c r="A208" s="4" t="n"/>
+      <c r="B208" s="4" t="n"/>
+      <c r="C208" s="4" t="n"/>
+      <c r="D208" s="4" t="n"/>
+      <c r="E208" s="4" t="n"/>
+      <c r="F208" s="4" t="n"/>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>PV 16 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="22" customHeight="1">
+      <c r="A209" s="4" t="n"/>
+      <c r="B209" s="4" t="n"/>
+      <c r="C209" s="4" t="n"/>
+      <c r="D209" s="4" t="n"/>
+      <c r="E209" s="4" t="n"/>
+      <c r="F209" s="4" t="n"/>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>PV 17 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="22" customHeight="1">
+      <c r="A210" s="4" t="n"/>
+      <c r="B210" s="4" t="n"/>
+      <c r="C210" s="4" t="n"/>
+      <c r="D210" s="4" t="n"/>
+      <c r="E210" s="4" t="n"/>
+      <c r="F210" s="4" t="n"/>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>PV 18 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="22" customHeight="1">
+      <c r="A211" s="4" t="n"/>
+      <c r="B211" s="4" t="n"/>
+      <c r="C211" s="4" t="n"/>
+      <c r="D211" s="4" t="n"/>
+      <c r="E211" s="4" t="n"/>
+      <c r="F211" s="4" t="n"/>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>PV 19 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="22" customHeight="1">
+      <c r="A212" s="4" t="n"/>
+      <c r="B212" s="4" t="n"/>
+      <c r="C212" s="4" t="n"/>
+      <c r="D212" s="4" t="n"/>
+      <c r="E212" s="4" t="n"/>
+      <c r="F212" s="4" t="n"/>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
           <t>PV 20 Current (A) String</t>
         </is>
       </c>
     </row>
-    <row r="200" ht="22" customHeight="1">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>SINCERELY DYEING</t>
-        </is>
-      </c>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="C200" s="2" t="n"/>
-      <c r="D200" s="2" t="inlineStr"/>
-      <c r="E200" s="2" t="inlineStr">
-        <is>
-          <t>TERA INV 5</t>
-        </is>
-      </c>
-      <c r="F200" s="2" t="inlineStr">
-        <is>
-          <t>ES24A0054424</t>
-        </is>
-      </c>
-      <c r="G200" s="2" t="inlineStr">
+    <row r="213" ht="22" customHeight="1">
+      <c r="A213" s="4" t="n"/>
+      <c r="B213" s="4" t="n"/>
+      <c r="C213" s="4" t="n"/>
+      <c r="D213" s="4" t="n"/>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_3</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>NE=53678487</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>PV 2 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="22" customHeight="1">
+      <c r="A214" s="4" t="n"/>
+      <c r="B214" s="4" t="n"/>
+      <c r="C214" s="4" t="n"/>
+      <c r="D214" s="4" t="n"/>
+      <c r="E214" s="4" t="n"/>
+      <c r="F214" s="4" t="n"/>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>PV 4 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="22" customHeight="1">
+      <c r="A215" s="4" t="n"/>
+      <c r="B215" s="4" t="n"/>
+      <c r="C215" s="4" t="n"/>
+      <c r="D215" s="4" t="n"/>
+      <c r="E215" s="4" t="n"/>
+      <c r="F215" s="4" t="n"/>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>PV 6 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="22" customHeight="1">
+      <c r="A216" s="4" t="n"/>
+      <c r="B216" s="4" t="n"/>
+      <c r="C216" s="4" t="n"/>
+      <c r="D216" s="4" t="n"/>
+      <c r="E216" s="4" t="n"/>
+      <c r="F216" s="4" t="n"/>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>PV 7 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="22" customHeight="1">
+      <c r="A217" s="4" t="n"/>
+      <c r="B217" s="4" t="n"/>
+      <c r="C217" s="4" t="n"/>
+      <c r="D217" s="4" t="n"/>
+      <c r="E217" s="4" t="n"/>
+      <c r="F217" s="4" t="n"/>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>PV 8 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="22" customHeight="1">
+      <c r="A218" s="4" t="n"/>
+      <c r="B218" s="4" t="n"/>
+      <c r="C218" s="4" t="n"/>
+      <c r="D218" s="4" t="n"/>
+      <c r="E218" s="4" t="n"/>
+      <c r="F218" s="4" t="n"/>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>PV 10 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="22" customHeight="1">
+      <c r="A219" s="4" t="n"/>
+      <c r="B219" s="4" t="n"/>
+      <c r="C219" s="4" t="n"/>
+      <c r="D219" s="4" t="n"/>
+      <c r="E219" s="4" t="n"/>
+      <c r="F219" s="4" t="n"/>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>PV 11 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="22" customHeight="1">
+      <c r="A220" s="4" t="n"/>
+      <c r="B220" s="4" t="n"/>
+      <c r="C220" s="4" t="n"/>
+      <c r="D220" s="4" t="n"/>
+      <c r="E220" s="4" t="n"/>
+      <c r="F220" s="4" t="n"/>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>PV 12 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="22" customHeight="1">
+      <c r="A221" s="4" t="n"/>
+      <c r="B221" s="4" t="n"/>
+      <c r="C221" s="4" t="n"/>
+      <c r="D221" s="4" t="n"/>
+      <c r="E221" s="4" t="n"/>
+      <c r="F221" s="4" t="n"/>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>PV 14 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="22" customHeight="1">
+      <c r="A222" s="4" t="n"/>
+      <c r="B222" s="4" t="n"/>
+      <c r="C222" s="4" t="n"/>
+      <c r="D222" s="4" t="n"/>
+      <c r="E222" s="4" t="n"/>
+      <c r="F222" s="4" t="n"/>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>PV 16 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="22" customHeight="1">
+      <c r="A223" s="4" t="n"/>
+      <c r="B223" s="4" t="n"/>
+      <c r="C223" s="4" t="n"/>
+      <c r="D223" s="4" t="n"/>
+      <c r="E223" s="4" t="n"/>
+      <c r="F223" s="4" t="n"/>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>PV 18 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="22" customHeight="1">
+      <c r="A224" s="4" t="n"/>
+      <c r="B224" s="4" t="n"/>
+      <c r="C224" s="4" t="n"/>
+      <c r="D224" s="4" t="n"/>
+      <c r="E224" s="4" t="n"/>
+      <c r="F224" s="4" t="n"/>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>PV 20 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="22" customHeight="1">
+      <c r="A225" s="4" t="n"/>
+      <c r="B225" s="4" t="n"/>
+      <c r="C225" s="4" t="n"/>
+      <c r="D225" s="4" t="n"/>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_4</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>NE=53678481</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>PV 2 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="22" customHeight="1">
+      <c r="A226" s="4" t="n"/>
+      <c r="B226" s="4" t="n"/>
+      <c r="C226" s="4" t="n"/>
+      <c r="D226" s="4" t="n"/>
+      <c r="E226" s="4" t="n"/>
+      <c r="F226" s="4" t="n"/>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>PV 9 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="22" customHeight="1">
+      <c r="A227" s="4" t="n"/>
+      <c r="B227" s="4" t="n"/>
+      <c r="C227" s="4" t="n"/>
+      <c r="D227" s="4" t="n"/>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_6</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>NE=53678483</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>PV 2 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="22" customHeight="1">
+      <c r="A228" s="4" t="n"/>
+      <c r="B228" s="4" t="n"/>
+      <c r="C228" s="4" t="n"/>
+      <c r="D228" s="4" t="n"/>
+      <c r="E228" s="4" t="n"/>
+      <c r="F228" s="4" t="n"/>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>PV 4 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="22" customHeight="1">
+      <c r="A229" s="4" t="n"/>
+      <c r="B229" s="4" t="n"/>
+      <c r="C229" s="4" t="n"/>
+      <c r="D229" s="4" t="n"/>
+      <c r="E229" s="4" t="n"/>
+      <c r="F229" s="4" t="n"/>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>PV 6 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="22" customHeight="1">
+      <c r="A230" s="4" t="n"/>
+      <c r="B230" s="4" t="n"/>
+      <c r="C230" s="4" t="n"/>
+      <c r="D230" s="4" t="n"/>
+      <c r="E230" s="4" t="n"/>
+      <c r="F230" s="4" t="n"/>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>PV 8 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="22" customHeight="1">
+      <c r="A231" s="4" t="n"/>
+      <c r="B231" s="4" t="n"/>
+      <c r="C231" s="4" t="n"/>
+      <c r="D231" s="4" t="n"/>
+      <c r="E231" s="4" t="n"/>
+      <c r="F231" s="4" t="n"/>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>PV 10 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="22" customHeight="1">
+      <c r="A232" s="4" t="n"/>
+      <c r="B232" s="4" t="n"/>
+      <c r="C232" s="4" t="n"/>
+      <c r="D232" s="4" t="n"/>
+      <c r="E232" s="4" t="n"/>
+      <c r="F232" s="4" t="n"/>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>PV 12 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="22" customHeight="1">
+      <c r="A233" s="4" t="n"/>
+      <c r="B233" s="4" t="n"/>
+      <c r="C233" s="4" t="n"/>
+      <c r="D233" s="4" t="n"/>
+      <c r="E233" s="4" t="n"/>
+      <c r="F233" s="4" t="n"/>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>PV 14 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="22" customHeight="1">
+      <c r="A234" s="4" t="n"/>
+      <c r="B234" s="4" t="n"/>
+      <c r="C234" s="4" t="n"/>
+      <c r="D234" s="4" t="n"/>
+      <c r="E234" s="4" t="n"/>
+      <c r="F234" s="4" t="n"/>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>PV 15 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="22" customHeight="1">
+      <c r="A235" s="4" t="n"/>
+      <c r="B235" s="4" t="n"/>
+      <c r="C235" s="4" t="n"/>
+      <c r="D235" s="4" t="n"/>
+      <c r="E235" s="4" t="n"/>
+      <c r="F235" s="4" t="n"/>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>PV 16 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="22" customHeight="1">
+      <c r="A236" s="4" t="n"/>
+      <c r="B236" s="4" t="n"/>
+      <c r="C236" s="4" t="n"/>
+      <c r="D236" s="4" t="n"/>
+      <c r="E236" s="4" t="n"/>
+      <c r="F236" s="4" t="n"/>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>PV 18 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="22" customHeight="1">
+      <c r="A237" s="4" t="n"/>
+      <c r="B237" s="4" t="n"/>
+      <c r="C237" s="4" t="n"/>
+      <c r="D237" s="4" t="n"/>
+      <c r="E237" s="4" t="n"/>
+      <c r="F237" s="4" t="n"/>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>PV 20 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="22" customHeight="1">
+      <c r="A238" s="4" t="n"/>
+      <c r="B238" s="4" t="n"/>
+      <c r="C238" s="4" t="n"/>
+      <c r="D238" s="4" t="n"/>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_7</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>NE=53676713</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>PV 2 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="22" customHeight="1">
+      <c r="A239" s="4" t="n"/>
+      <c r="B239" s="4" t="n"/>
+      <c r="C239" s="4" t="n"/>
+      <c r="D239" s="4" t="n"/>
+      <c r="E239" s="4" t="n"/>
+      <c r="F239" s="4" t="n"/>
+      <c r="G239" s="2" t="inlineStr">
         <is>
           <t>PV 5 Current (A) String</t>
         </is>
       </c>
     </row>
+    <row r="240" ht="22" customHeight="1">
+      <c r="A240" s="4" t="n"/>
+      <c r="B240" s="4" t="n"/>
+      <c r="C240" s="4" t="n"/>
+      <c r="D240" s="4" t="n"/>
+      <c r="E240" s="4" t="n"/>
+      <c r="F240" s="4" t="n"/>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>PV 6 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="22" customHeight="1">
+      <c r="A241" s="4" t="n"/>
+      <c r="B241" s="4" t="n"/>
+      <c r="C241" s="4" t="n"/>
+      <c r="D241" s="4" t="n"/>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>INVERTER_9</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>NE=53679667</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>PV 1 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="22" customHeight="1">
+      <c r="A242" s="4" t="n"/>
+      <c r="B242" s="4" t="n"/>
+      <c r="C242" s="4" t="n"/>
+      <c r="D242" s="4" t="n"/>
+      <c r="E242" s="4" t="n"/>
+      <c r="F242" s="4" t="n"/>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>PV 2 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="22" customHeight="1">
+      <c r="A243" s="4" t="n"/>
+      <c r="B243" s="4" t="n"/>
+      <c r="C243" s="4" t="n"/>
+      <c r="D243" s="4" t="n"/>
+      <c r="E243" s="4" t="n"/>
+      <c r="F243" s="4" t="n"/>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>PV 3 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="22" customHeight="1">
+      <c r="A244" s="4" t="n"/>
+      <c r="B244" s="4" t="n"/>
+      <c r="C244" s="4" t="n"/>
+      <c r="D244" s="4" t="n"/>
+      <c r="E244" s="4" t="n"/>
+      <c r="F244" s="4" t="n"/>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>PV 4 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="22" customHeight="1">
+      <c r="A245" s="4" t="n"/>
+      <c r="B245" s="4" t="n"/>
+      <c r="C245" s="4" t="n"/>
+      <c r="D245" s="4" t="n"/>
+      <c r="E245" s="4" t="n"/>
+      <c r="F245" s="4" t="n"/>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>PV 6 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="22" customHeight="1">
+      <c r="A246" s="4" t="n"/>
+      <c r="B246" s="4" t="n"/>
+      <c r="C246" s="4" t="n"/>
+      <c r="D246" s="4" t="n"/>
+      <c r="E246" s="4" t="n"/>
+      <c r="F246" s="4" t="n"/>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>PV 7 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="22" customHeight="1">
+      <c r="A247" s="4" t="n"/>
+      <c r="B247" s="4" t="n"/>
+      <c r="C247" s="4" t="n"/>
+      <c r="D247" s="4" t="n"/>
+      <c r="E247" s="4" t="n"/>
+      <c r="F247" s="4" t="n"/>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>PV 8 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="22" customHeight="1">
+      <c r="A248" s="4" t="n"/>
+      <c r="B248" s="4" t="n"/>
+      <c r="C248" s="4" t="n"/>
+      <c r="D248" s="4" t="n"/>
+      <c r="E248" s="4" t="n"/>
+      <c r="F248" s="4" t="n"/>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>PV 9 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="22" customHeight="1">
+      <c r="A249" s="4" t="n"/>
+      <c r="B249" s="4" t="n"/>
+      <c r="C249" s="4" t="n"/>
+      <c r="D249" s="4" t="n"/>
+      <c r="E249" s="4" t="n"/>
+      <c r="F249" s="4" t="n"/>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>PV 10 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="22" customHeight="1">
+      <c r="A250" s="4" t="n"/>
+      <c r="B250" s="4" t="n"/>
+      <c r="C250" s="4" t="n"/>
+      <c r="D250" s="4" t="n"/>
+      <c r="E250" s="4" t="n"/>
+      <c r="F250" s="4" t="n"/>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>PV 11 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="22" customHeight="1">
+      <c r="A251" s="4" t="n"/>
+      <c r="B251" s="4" t="n"/>
+      <c r="C251" s="4" t="n"/>
+      <c r="D251" s="4" t="n"/>
+      <c r="E251" s="4" t="n"/>
+      <c r="F251" s="4" t="n"/>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>PV 12 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="22" customHeight="1">
+      <c r="A252" s="4" t="n"/>
+      <c r="B252" s="4" t="n"/>
+      <c r="C252" s="4" t="n"/>
+      <c r="D252" s="4" t="n"/>
+      <c r="E252" s="4" t="n"/>
+      <c r="F252" s="4" t="n"/>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>PV 13 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="22" customHeight="1">
+      <c r="A253" s="4" t="n"/>
+      <c r="B253" s="4" t="n"/>
+      <c r="C253" s="4" t="n"/>
+      <c r="D253" s="4" t="n"/>
+      <c r="E253" s="4" t="n"/>
+      <c r="F253" s="4" t="n"/>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>PV 14 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="22" customHeight="1">
+      <c r="A254" s="4" t="n"/>
+      <c r="B254" s="4" t="n"/>
+      <c r="C254" s="4" t="n"/>
+      <c r="D254" s="4" t="n"/>
+      <c r="E254" s="4" t="n"/>
+      <c r="F254" s="4" t="n"/>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>PV 15 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="22" customHeight="1">
+      <c r="A255" s="4" t="n"/>
+      <c r="B255" s="4" t="n"/>
+      <c r="C255" s="4" t="n"/>
+      <c r="D255" s="4" t="n"/>
+      <c r="E255" s="4" t="n"/>
+      <c r="F255" s="4" t="n"/>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>PV 16 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="22" customHeight="1">
+      <c r="A256" s="4" t="n"/>
+      <c r="B256" s="4" t="n"/>
+      <c r="C256" s="4" t="n"/>
+      <c r="D256" s="4" t="n"/>
+      <c r="E256" s="4" t="n"/>
+      <c r="F256" s="4" t="n"/>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>PV 17 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="22" customHeight="1">
+      <c r="A257" s="4" t="n"/>
+      <c r="B257" s="4" t="n"/>
+      <c r="C257" s="4" t="n"/>
+      <c r="D257" s="4" t="n"/>
+      <c r="E257" s="4" t="n"/>
+      <c r="F257" s="4" t="n"/>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>PV 18 Current (A) String</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="22" customHeight="1">
+      <c r="A258" s="4" t="n"/>
+      <c r="B258" s="4" t="n"/>
+      <c r="C258" s="4" t="n"/>
+      <c r="D258" s="4" t="n"/>
+      <c r="E258" s="4" t="n"/>
+      <c r="F258" s="4" t="n"/>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>PV 20 Current (A) String</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="52">
-    <mergeCell ref="A31:A199"/>
-    <mergeCell ref="B31:B199"/>
-    <mergeCell ref="E31:E48"/>
-    <mergeCell ref="E91:E109"/>
-    <mergeCell ref="D31:D199"/>
-    <mergeCell ref="F31:F48"/>
-    <mergeCell ref="E179:E181"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E129:E134"/>
-    <mergeCell ref="F68:F71"/>
-    <mergeCell ref="E135:E153"/>
-    <mergeCell ref="F10:F15"/>
-    <mergeCell ref="F164:F165"/>
-    <mergeCell ref="E182:E199"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="A26:A30"/>
-    <mergeCell ref="F179:F181"/>
-    <mergeCell ref="F16:F23"/>
-    <mergeCell ref="C10:C24"/>
-    <mergeCell ref="E166:E178"/>
-    <mergeCell ref="E10:E15"/>
-    <mergeCell ref="F129:F134"/>
+  <mergeCells count="66">
+    <mergeCell ref="F227:F237"/>
+    <mergeCell ref="E106:E124"/>
+    <mergeCell ref="D88:D258"/>
+    <mergeCell ref="F66:F72"/>
+    <mergeCell ref="E61:E65"/>
+    <mergeCell ref="F38:F42"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E31:E37"/>
+    <mergeCell ref="E194:E212"/>
+    <mergeCell ref="E188:E193"/>
+    <mergeCell ref="F31:F37"/>
+    <mergeCell ref="A88:A258"/>
+    <mergeCell ref="B13:B87"/>
+    <mergeCell ref="E241:E258"/>
+    <mergeCell ref="E150:E168"/>
+    <mergeCell ref="D13:D87"/>
+    <mergeCell ref="E21:E30"/>
+    <mergeCell ref="F61:F65"/>
+    <mergeCell ref="E66:E72"/>
+    <mergeCell ref="E131:E149"/>
+    <mergeCell ref="C11:C12"/>
     <mergeCell ref="B2:B9"/>
+    <mergeCell ref="C88:C258"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F73:F79"/>
+    <mergeCell ref="F80:F87"/>
+    <mergeCell ref="E213:E224"/>
+    <mergeCell ref="E238:E240"/>
     <mergeCell ref="D2:D9"/>
-    <mergeCell ref="C31:C199"/>
-    <mergeCell ref="E68:E71"/>
-    <mergeCell ref="D10:D24"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="F110:F128"/>
-    <mergeCell ref="D26:D30"/>
-    <mergeCell ref="F182:F199"/>
+    <mergeCell ref="E225:E226"/>
+    <mergeCell ref="F43:F51"/>
+    <mergeCell ref="E13:E20"/>
+    <mergeCell ref="F194:F212"/>
+    <mergeCell ref="F188:F193"/>
+    <mergeCell ref="F52:F60"/>
+    <mergeCell ref="A13:A87"/>
+    <mergeCell ref="C13:C87"/>
+    <mergeCell ref="F241:F258"/>
+    <mergeCell ref="B88:B258"/>
+    <mergeCell ref="F150:F168"/>
+    <mergeCell ref="F21:F30"/>
+    <mergeCell ref="F88:F105"/>
     <mergeCell ref="F2:F9"/>
-    <mergeCell ref="F91:F109"/>
-    <mergeCell ref="F135:F153"/>
-    <mergeCell ref="B10:B24"/>
-    <mergeCell ref="F72:F90"/>
-    <mergeCell ref="E49:E67"/>
-    <mergeCell ref="F154:F163"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="C26:C30"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="E110:E128"/>
-    <mergeCell ref="F166:F178"/>
+    <mergeCell ref="F131:F149"/>
+    <mergeCell ref="F169:F187"/>
+    <mergeCell ref="F125:F130"/>
+    <mergeCell ref="E73:E79"/>
+    <mergeCell ref="E80:E87"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E43:E51"/>
+    <mergeCell ref="E227:E237"/>
+    <mergeCell ref="F238:F240"/>
+    <mergeCell ref="F13:F20"/>
+    <mergeCell ref="E52:E60"/>
+    <mergeCell ref="F106:F124"/>
     <mergeCell ref="A2:A9"/>
+    <mergeCell ref="E88:E105"/>
     <mergeCell ref="C2:C9"/>
+    <mergeCell ref="F213:F224"/>
     <mergeCell ref="E2:E9"/>
-    <mergeCell ref="A10:A24"/>
-    <mergeCell ref="E164:E165"/>
-    <mergeCell ref="E72:E90"/>
-    <mergeCell ref="E16:E23"/>
-    <mergeCell ref="E154:E163"/>
-    <mergeCell ref="F49:F67"/>
+    <mergeCell ref="E38:E42"/>
+    <mergeCell ref="E169:E187"/>
+    <mergeCell ref="F225:F226"/>
+    <mergeCell ref="E125:E130"/>
+    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>